<commit_message>
Add CR1-review, Analisis: Cambios_vs_Prioridad
Revisión y completado de las solicitudes de cambio. y realización del analisis de prioridad.
</commit_message>
<xml_diff>
--- a/documentation/Construccion y Evolucion/1. Solicitudes de cambio/CR 1.xlsx
+++ b/documentation/Construccion y Evolucion/1. Solicitudes de cambio/CR 1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Proyectos\TraductorBraille\documentation\Construccion y Evolucion\1. Solicitudes de cambio\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\translator\TraductorBrailleEspanol\documentation\Construccion y Evolucion\1. Solicitudes de cambio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD3ED88D-D6C7-4F50-A325-9EC27D74204C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08274585-19A0-4710-A613-337F19E2BDDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11040" xr2:uid="{AAACD53E-982C-4521-B07F-7DC6290E23F5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" firstSheet="1" activeTab="1" xr2:uid="{AAACD53E-982C-4521-B07F-7DC6290E23F5}"/>
   </bookViews>
   <sheets>
     <sheet name="CR Formato" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="52">
   <si>
     <t>CHANGE REQUEST</t>
   </si>
@@ -152,6 +152,38 @@
   </si>
   <si>
     <t>Christian Nazate</t>
+  </si>
+  <si>
+    <t>SofTech</t>
+  </si>
+  <si>
+    <t>Brailingo - SoftTech</t>
+  </si>
+  <si>
+    <t>1. Utilizar java.io para leer archivos TXT y Apache PDFBox para extraer texto de PDFs.
+2. Integrar una librería o servicio externo especializado en la traducción de archivos, 
+3.Desarrollar métodos internos para manejar la carga y traducción de archivos según su tipo</t>
+  </si>
+  <si>
+    <t>Utilizar la opción de java.io junto con Apache PDFBox, ya que es una solución sencilla, de fácil integración en Java, y te proporciona control sobre el procesamiento de archivos TXT y PDF sin depender de servicios externos.</t>
+  </si>
+  <si>
+    <t>GUI</t>
+  </si>
+  <si>
+    <t>Añadir Opción de importación</t>
+  </si>
+  <si>
+    <t>Class Import</t>
+  </si>
+  <si>
+    <t>Añadir un clase para implementar la lógica.</t>
+  </si>
+  <si>
+    <t>Medio</t>
+  </si>
+  <si>
+    <t>2 dias</t>
   </si>
 </sst>
 </file>
@@ -442,7 +474,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -516,22 +548,43 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -868,7 +921,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F84A08-0160-4953-9528-DB07A5F993CD}">
   <dimension ref="B1:H33"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="5.5703125" customWidth="1"/>
     <col min="3" max="3" width="36.42578125" bestFit="1" customWidth="1"/>
@@ -1040,8 +1093,12 @@
         <v>13</v>
       </c>
       <c r="D20" s="9"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="8"/>
+      <c r="E20" s="10">
+        <v>45517</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>42</v>
+      </c>
       <c r="G20" s="8"/>
       <c r="H20" s="7"/>
     </row>
@@ -1051,8 +1108,12 @@
         <v>14</v>
       </c>
       <c r="D21" s="9"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="8"/>
+      <c r="E21" s="10">
+        <v>45517</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>42</v>
+      </c>
       <c r="G21" s="8"/>
       <c r="H21" s="7"/>
     </row>
@@ -1062,8 +1123,12 @@
         <v>15</v>
       </c>
       <c r="D22" s="9"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
+      <c r="E22" s="10">
+        <v>45517</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>42</v>
+      </c>
       <c r="G22" s="8"/>
       <c r="H22" s="7"/>
     </row>
@@ -1189,7 +1254,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33198599-D7F8-440A-9813-85D60D291D95}">
   <dimension ref="B1:H34"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.5703125" customWidth="1"/>
     <col min="3" max="3" width="39" bestFit="1" customWidth="1"/>
@@ -1244,7 +1309,9 @@
       <c r="C7" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="37"/>
+      <c r="D7" s="37" t="s">
+        <v>43</v>
+      </c>
       <c r="E7" s="37"/>
       <c r="F7" s="37"/>
       <c r="G7" s="37"/>
@@ -1267,7 +1334,9 @@
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="4"/>
-      <c r="C10" s="38"/>
+      <c r="C10" s="38" t="s">
+        <v>44</v>
+      </c>
       <c r="D10" s="39"/>
       <c r="E10" s="39"/>
       <c r="F10" s="39"/>
@@ -1336,8 +1405,12 @@
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="4"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="34"/>
+      <c r="C18" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" s="34" t="s">
+        <v>47</v>
+      </c>
       <c r="E18" s="35"/>
       <c r="F18" s="35"/>
       <c r="G18" s="36"/>
@@ -1345,8 +1418,12 @@
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="4"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="34"/>
+      <c r="C19" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="34" t="s">
+        <v>49</v>
+      </c>
       <c r="E19" s="35"/>
       <c r="F19" s="35"/>
       <c r="G19" s="36"/>
@@ -1372,8 +1449,8 @@
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" s="4"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="39"/>
+      <c r="F22" s="44"/>
+      <c r="G22" s="44"/>
       <c r="H22" s="7"/>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.25">
@@ -1381,7 +1458,9 @@
       <c r="C23" t="s">
         <v>32</v>
       </c>
-      <c r="D23" s="17"/>
+      <c r="D23" s="17" t="s">
+        <v>51</v>
+      </c>
       <c r="H23" s="7"/>
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.25">
@@ -1392,6 +1471,9 @@
       <c r="B25" s="4"/>
       <c r="C25" t="s">
         <v>33</v>
+      </c>
+      <c r="D25" t="s">
+        <v>50</v>
       </c>
       <c r="H25" s="7"/>
     </row>
@@ -1420,47 +1502,49 @@
     </row>
     <row r="29" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B29" s="4"/>
-      <c r="C29" s="38"/>
-      <c r="D29" s="39"/>
-      <c r="E29" s="39"/>
-      <c r="F29" s="39"/>
-      <c r="G29" s="40"/>
+      <c r="C29" s="45" t="s">
+        <v>45</v>
+      </c>
+      <c r="D29" s="46"/>
+      <c r="E29" s="46"/>
+      <c r="F29" s="46"/>
+      <c r="G29" s="47"/>
       <c r="H29" s="7"/>
     </row>
     <row r="30" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B30" s="4"/>
-      <c r="C30" s="38"/>
-      <c r="D30" s="39"/>
-      <c r="E30" s="39"/>
-      <c r="F30" s="39"/>
-      <c r="G30" s="40"/>
+      <c r="C30" s="45"/>
+      <c r="D30" s="46"/>
+      <c r="E30" s="46"/>
+      <c r="F30" s="46"/>
+      <c r="G30" s="47"/>
       <c r="H30" s="7"/>
     </row>
     <row r="31" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B31" s="4"/>
-      <c r="C31" s="38"/>
-      <c r="D31" s="39"/>
-      <c r="E31" s="39"/>
-      <c r="F31" s="39"/>
-      <c r="G31" s="40"/>
+      <c r="C31" s="45"/>
+      <c r="D31" s="46"/>
+      <c r="E31" s="46"/>
+      <c r="F31" s="46"/>
+      <c r="G31" s="47"/>
       <c r="H31" s="7"/>
     </row>
     <row r="32" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B32" s="4"/>
-      <c r="C32" s="38"/>
-      <c r="D32" s="39"/>
-      <c r="E32" s="39"/>
-      <c r="F32" s="39"/>
-      <c r="G32" s="40"/>
+      <c r="C32" s="45"/>
+      <c r="D32" s="46"/>
+      <c r="E32" s="46"/>
+      <c r="F32" s="46"/>
+      <c r="G32" s="47"/>
       <c r="H32" s="7"/>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" s="4"/>
-      <c r="C33" s="41"/>
-      <c r="D33" s="42"/>
-      <c r="E33" s="42"/>
-      <c r="F33" s="42"/>
-      <c r="G33" s="43"/>
+      <c r="C33" s="48"/>
+      <c r="D33" s="49"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="49"/>
+      <c r="G33" s="50"/>
       <c r="H33" s="7"/>
     </row>
     <row r="34" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1489,20 +1573,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="f7b1a7ea-1dd0-43bd-8f52-dd9459d0ec96" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="f7b1a7ea-1dd0-43bd-8f52-dd9459d0ec96" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1753,6 +1837,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3BE880B-0D64-411C-BD75-74863A321A9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{96BACB75-2D9E-4BF9-B15E-EA86EAB29BB3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -1765,14 +1857,6 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="56eae398-d265-4f71-b30c-62c529056c9f"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3BE880B-0D64-411C-BD75-74863A321A9B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>